<commit_message>
archivos actualizados a 22 septiembre
</commit_message>
<xml_diff>
--- a/originales/respuestas/2025/01. Calificadas/root/Alcaldía Local De Barrios Unidos.xlsx
+++ b/originales/respuestas/2025/01. Calificadas/root/Alcaldía Local De Barrios Unidos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Personal\Desktop\Respuesta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{891291A2-C9A7-492C-BE79-8061AC13913F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E73C021-C572-46A6-AD73-8E07AAA5DC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{61CCE0CF-AD1F-450B-B0AC-9AFFE8214C2E}"/>
+    <workbookView xWindow="3075" yWindow="0" windowWidth="23040" windowHeight="15480" activeTab="4" xr2:uid="{61CCE0CF-AD1F-450B-B0AC-9AFFE8214C2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1564,7 +1564,7 @@
         <v>42</v>
       </c>
       <c r="S7" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
@@ -1634,7 +1634,7 @@
         <v>30</v>
       </c>
       <c r="S8" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T8" s="8"/>
       <c r="U8" s="8"/>
@@ -1680,7 +1680,7 @@
         <v>38</v>
       </c>
       <c r="K9" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>39</v>
@@ -1746,7 +1746,7 @@
         <v>38</v>
       </c>
       <c r="K10" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>39</v>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="J11" s="6"/>
       <c r="K11" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L11" s="6"/>
       <c r="M11" s="6">
@@ -1886,7 +1886,7 @@
         <v>42</v>
       </c>
       <c r="S12" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T12" s="8"/>
       <c r="U12" s="8"/>
@@ -2006,7 +2006,7 @@
         <v>42</v>
       </c>
       <c r="S14" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T14" s="8"/>
       <c r="U14" s="8"/>
@@ -2052,19 +2052,19 @@
         <v>38</v>
       </c>
       <c r="K15" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L15" s="9" t="s">
         <v>39</v>
       </c>
       <c r="M15" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N15" s="9" t="s">
         <v>40</v>
       </c>
       <c r="O15" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P15" s="9" t="s">
         <v>41</v>
@@ -2118,19 +2118,19 @@
         <v>38</v>
       </c>
       <c r="K16" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L16" s="9" t="s">
         <v>39</v>
       </c>
       <c r="M16" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N16" s="9" t="s">
         <v>40</v>
       </c>
       <c r="O16" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P16" s="9" t="s">
         <v>41</v>
@@ -2618,25 +2618,25 @@
         <v>26</v>
       </c>
       <c r="K2" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L2" s="12" t="s">
         <v>27</v>
       </c>
       <c r="M2" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N2" s="6" t="s">
         <v>28</v>
       </c>
       <c r="O2" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P2" s="6" t="s">
         <v>29</v>
       </c>
       <c r="Q2" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R2" s="6" t="s">
         <v>30</v>
@@ -2909,7 +2909,7 @@
       </c>
       <c r="L7" s="12"/>
       <c r="M7" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6"/>
       <c r="O7" s="6">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="L8" s="12"/>
       <c r="M8" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N8" s="6"/>
       <c r="O8" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P8" s="6"/>
       <c r="Q8" s="6">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="R8" s="6"/>
       <c r="S8" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:30" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="L9" s="14"/>
       <c r="M9" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N9" s="9"/>
       <c r="O9" s="9">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="L10" s="14"/>
       <c r="M10" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" s="9"/>
       <c r="O10" s="9">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="J11" s="6"/>
       <c r="K11" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L11" s="12"/>
       <c r="M11" s="6">
@@ -3109,11 +3109,11 @@
       </c>
       <c r="N11" s="6"/>
       <c r="O11" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P11" s="6"/>
       <c r="Q11" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R11" s="6"/>
       <c r="S11" s="6">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="L15" s="12"/>
       <c r="M15" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N15" s="6"/>
       <c r="O15" s="6">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="P15" s="6"/>
       <c r="Q15" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R15" s="6"/>
       <c r="S15" s="6">
@@ -3348,7 +3348,7 @@
         <v>26</v>
       </c>
       <c r="K16" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L16" s="12" t="s">
         <v>27</v>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="N19" s="6"/>
       <c r="O19" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P19" s="6"/>
       <c r="Q19" s="6">
@@ -3922,23 +3922,23 @@
       </c>
       <c r="J3" s="16"/>
       <c r="K3" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L3" s="17"/>
       <c r="M3" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N3" s="16"/>
       <c r="O3" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P3" s="16"/>
       <c r="Q3" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R3" s="16"/>
       <c r="S3" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3967,23 +3967,23 @@
       </c>
       <c r="J4" s="16"/>
       <c r="K4" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L4" s="17"/>
       <c r="M4" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4" s="16"/>
       <c r="O4" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P4" s="16"/>
       <c r="Q4" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R4" s="16"/>
       <c r="S4" s="16">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:31" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>